<commit_message>
week 7s work and updating hours
</commit_message>
<xml_diff>
--- a/Documentation/F25/JustinHours.xlsx
+++ b/Documentation/F25/JustinHours.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juxin\Documents\MIDI-Projects\Documentation\F25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E86C0DF0-F399-42F0-8072-1B60C2D838C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F0ACDC3-1C60-4484-947E-3AECE2FD3171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="32">
   <si>
     <t>Date</t>
   </si>
@@ -123,6 +123,15 @@
   </si>
   <si>
     <t>Physical design</t>
+  </si>
+  <si>
+    <t>Mechanical drawings write up</t>
+  </si>
+  <si>
+    <t>Infrared write up</t>
+  </si>
+  <si>
+    <t>Physical construction</t>
   </si>
 </sst>
 </file>
@@ -274,9 +283,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -286,14 +292,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -700,10 +709,10 @@
         <v>9</v>
       </c>
       <c r="T6" s="12"/>
-      <c r="U6" s="21" t="s">
+      <c r="U6" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="V6" s="22"/>
+      <c r="V6" s="20"/>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
@@ -731,8 +740,8 @@
       <c r="K7" s="12"/>
       <c r="S7" s="12"/>
       <c r="T7" s="12"/>
-      <c r="U7" s="22"/>
-      <c r="V7" s="22"/>
+      <c r="U7" s="20"/>
+      <c r="V7" s="20"/>
     </row>
     <row r="8" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
@@ -758,14 +767,14 @@
       <c r="I8" s="12"/>
       <c r="J8" s="12"/>
       <c r="K8" s="12"/>
-      <c r="S8" s="16" t="s">
+      <c r="S8" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="T8" s="16"/>
-      <c r="U8" s="16">
+      <c r="T8" s="21"/>
+      <c r="U8" s="21">
         <v>430450810</v>
       </c>
-      <c r="V8" s="16"/>
+      <c r="V8" s="21"/>
     </row>
     <row r="9" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
@@ -791,14 +800,14 @@
       <c r="I9" s="12"/>
       <c r="J9" s="12"/>
       <c r="K9" s="12"/>
-      <c r="S9" s="16" t="s">
+      <c r="S9" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="T9" s="16"/>
-      <c r="U9" s="16">
+      <c r="T9" s="21"/>
+      <c r="U9" s="21">
         <v>430450200</v>
       </c>
-      <c r="V9" s="16"/>
+      <c r="V9" s="21"/>
     </row>
     <row r="10" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
@@ -875,13 +884,13 @@
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="J12" s="20"/>
-      <c r="K12" s="20"/>
+      <c r="H12" s="22"/>
+      <c r="I12" s="22"/>
+      <c r="J12" s="22"/>
+      <c r="K12" s="22"/>
       <c r="R12" s="6"/>
       <c r="S12" s="7"/>
       <c r="T12" s="7"/>
@@ -907,13 +916,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G13" s="20" t="s">
+      <c r="G13" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
-      <c r="J13" s="20"/>
-      <c r="K13" s="20"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="22"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="22"/>
       <c r="S13"/>
       <c r="T13"/>
       <c r="U13"/>
@@ -936,13 +945,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G14" s="20" t="s">
+      <c r="G14" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
-      <c r="J14" s="20"/>
-      <c r="K14" s="20"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="22"/>
+      <c r="J14" s="22"/>
+      <c r="K14" s="22"/>
       <c r="S14"/>
       <c r="T14"/>
       <c r="U14"/>
@@ -965,13 +974,13 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999982</v>
       </c>
-      <c r="G15" s="20" t="s">
+      <c r="G15" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="J15" s="20"/>
-      <c r="K15" s="20"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="22"/>
+      <c r="J15" s="22"/>
+      <c r="K15" s="22"/>
       <c r="S15"/>
       <c r="T15"/>
       <c r="U15"/>
@@ -994,13 +1003,13 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G16" s="20" t="s">
+      <c r="G16" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="22"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
       <c r="S16"/>
       <c r="T16"/>
       <c r="U16"/>
@@ -1023,13 +1032,13 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999996</v>
       </c>
-      <c r="G17" s="20" t="s">
+      <c r="G17" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="H17" s="20"/>
-      <c r="I17" s="20"/>
-      <c r="J17" s="20"/>
-      <c r="K17" s="20"/>
+      <c r="H17" s="22"/>
+      <c r="I17" s="22"/>
+      <c r="J17" s="22"/>
+      <c r="K17" s="22"/>
       <c r="S17"/>
       <c r="T17"/>
       <c r="U17"/>
@@ -1052,13 +1061,13 @@
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="G18" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="H18" s="20"/>
-      <c r="I18" s="20"/>
-      <c r="J18" s="20"/>
-      <c r="K18" s="20"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="22"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="22"/>
       <c r="S18"/>
       <c r="T18"/>
       <c r="U18"/>
@@ -1081,13 +1090,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G19" s="20" t="s">
+      <c r="G19" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
-      <c r="J19" s="20"/>
-      <c r="K19" s="20"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="22"/>
+      <c r="K19" s="22"/>
       <c r="S19"/>
       <c r="T19"/>
       <c r="U19"/>
@@ -1110,13 +1119,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G20" s="20" t="s">
+      <c r="G20" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="H20" s="20"/>
-      <c r="I20" s="20"/>
-      <c r="J20" s="20"/>
-      <c r="K20" s="20"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
       <c r="S20"/>
       <c r="T20"/>
       <c r="U20"/>
@@ -1139,13 +1148,13 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999982</v>
       </c>
-      <c r="G21" s="20" t="s">
+      <c r="G21" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="H21" s="20"/>
-      <c r="I21" s="20"/>
-      <c r="J21" s="20"/>
-      <c r="K21" s="20"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
     </row>
     <row r="22" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B22" s="2">
@@ -1289,13 +1298,13 @@
         <f t="shared" si="0"/>
         <v>2.333333333333333</v>
       </c>
-      <c r="G27" s="17" t="s">
+      <c r="G27" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="H27" s="18"/>
-      <c r="I27" s="18"/>
-      <c r="J27" s="18"/>
-      <c r="K27" s="19"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="18"/>
     </row>
     <row r="28" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B28" s="2">
@@ -1314,13 +1323,13 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G28" s="17" t="s">
+      <c r="G28" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="18"/>
-      <c r="K28" s="19"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="18"/>
     </row>
     <row r="29" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B29" s="2">
@@ -1339,13 +1348,13 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G29" s="17" t="s">
+      <c r="G29" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="H29" s="18"/>
-      <c r="I29" s="18"/>
-      <c r="J29" s="18"/>
-      <c r="K29" s="19"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="18"/>
     </row>
     <row r="30" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B30" s="2">
@@ -1364,13 +1373,13 @@
         <f t="shared" ref="F30:F45" si="1">ABS((E30-D30)*24)</f>
         <v>3</v>
       </c>
-      <c r="G30" s="17" t="s">
+      <c r="G30" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="18"/>
-      <c r="I30" s="18"/>
-      <c r="J30" s="18"/>
-      <c r="K30" s="19"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="17"/>
+      <c r="J30" s="17"/>
+      <c r="K30" s="18"/>
     </row>
     <row r="31" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B31" s="2">
@@ -1389,13 +1398,13 @@
         <f t="shared" si="1"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G31" s="17" t="s">
+      <c r="G31" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
-      <c r="J31" s="18"/>
-      <c r="K31" s="19"/>
+      <c r="H31" s="17"/>
+      <c r="I31" s="17"/>
+      <c r="J31" s="17"/>
+      <c r="K31" s="18"/>
     </row>
     <row r="32" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B32" s="8">
@@ -1923,240 +1932,300 @@
       <c r="K52" s="12"/>
     </row>
     <row r="53" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B53" s="2">
+      <c r="B53" s="8">
         <v>6</v>
       </c>
-      <c r="C53" s="3">
+      <c r="C53" s="9">
         <v>45992</v>
       </c>
-      <c r="D53" s="4">
+      <c r="D53" s="10">
         <v>0.42708333333333331</v>
       </c>
-      <c r="E53" s="4">
+      <c r="E53" s="10">
         <v>0.5</v>
       </c>
-      <c r="F53" s="5">
+      <c r="F53" s="11">
         <f t="shared" si="2"/>
         <v>1.7500000000000004</v>
       </c>
-      <c r="G53" s="12" t="s">
+      <c r="G53" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="H53" s="12"/>
-      <c r="I53" s="12"/>
-      <c r="J53" s="12"/>
-      <c r="K53" s="12"/>
+      <c r="H53" s="22"/>
+      <c r="I53" s="22"/>
+      <c r="J53" s="22"/>
+      <c r="K53" s="22"/>
     </row>
     <row r="54" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B54" s="2">
+      <c r="B54" s="8">
         <v>6</v>
       </c>
-      <c r="C54" s="3">
+      <c r="C54" s="9">
         <v>45992</v>
       </c>
-      <c r="D54" s="4">
+      <c r="D54" s="10">
         <v>0.53125</v>
       </c>
-      <c r="E54" s="4">
+      <c r="E54" s="10">
         <v>0.56944444444444442</v>
       </c>
-      <c r="F54" s="5">
+      <c r="F54" s="11">
         <f t="shared" si="2"/>
         <v>0.91666666666666607</v>
       </c>
-      <c r="G54" s="12" t="s">
+      <c r="G54" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="H54" s="12"/>
-      <c r="I54" s="12"/>
-      <c r="J54" s="12"/>
-      <c r="K54" s="12"/>
+      <c r="H54" s="22"/>
+      <c r="I54" s="22"/>
+      <c r="J54" s="22"/>
+      <c r="K54" s="22"/>
     </row>
     <row r="55" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B55" s="2">
+      <c r="B55" s="8">
         <v>6</v>
       </c>
-      <c r="C55" s="3">
+      <c r="C55" s="9">
         <v>45992</v>
       </c>
-      <c r="D55" s="4"/>
-      <c r="E55" s="4"/>
-      <c r="F55" s="5">
+      <c r="D55" s="10">
+        <v>0.56944444444444442</v>
+      </c>
+      <c r="E55" s="10">
+        <v>0.61805555555555558</v>
+      </c>
+      <c r="F55" s="11">
         <f t="shared" ref="F55:F68" si="3">ABS((E55-D55)*24)</f>
-        <v>0</v>
-      </c>
-      <c r="G55" s="12"/>
-      <c r="H55" s="12"/>
-      <c r="I55" s="12"/>
-      <c r="J55" s="12"/>
-      <c r="K55" s="12"/>
+        <v>1.1666666666666679</v>
+      </c>
+      <c r="G55" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="H55" s="22"/>
+      <c r="I55" s="22"/>
+      <c r="J55" s="22"/>
+      <c r="K55" s="22"/>
     </row>
     <row r="56" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B56" s="2">
+      <c r="B56" s="8">
         <v>6</v>
       </c>
-      <c r="C56" s="3">
-        <v>45992</v>
-      </c>
-      <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
-      <c r="F56" s="5">
+      <c r="C56" s="9">
+        <v>45993</v>
+      </c>
+      <c r="D56" s="10">
+        <v>0.4375</v>
+      </c>
+      <c r="E56" s="10">
+        <v>0.49305555555555558</v>
+      </c>
+      <c r="F56" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G56" s="12"/>
-      <c r="H56" s="12"/>
-      <c r="I56" s="12"/>
-      <c r="J56" s="12"/>
-      <c r="K56" s="12"/>
+        <v>1.3333333333333339</v>
+      </c>
+      <c r="G56" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H56" s="22"/>
+      <c r="I56" s="22"/>
+      <c r="J56" s="22"/>
+      <c r="K56" s="22"/>
     </row>
     <row r="57" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B57" s="2">
+      <c r="B57" s="8">
         <v>6</v>
       </c>
-      <c r="C57" s="3">
-        <v>45992</v>
-      </c>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
-      <c r="F57" s="5">
+      <c r="C57" s="9">
+        <v>45993</v>
+      </c>
+      <c r="D57" s="10">
+        <v>0.53125</v>
+      </c>
+      <c r="E57" s="10">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F57" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G57" s="12"/>
-      <c r="H57" s="12"/>
-      <c r="I57" s="12"/>
-      <c r="J57" s="12"/>
-      <c r="K57" s="12"/>
+        <v>4.2500000000000009</v>
+      </c>
+      <c r="G57" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="H57" s="22"/>
+      <c r="I57" s="22"/>
+      <c r="J57" s="22"/>
+      <c r="K57" s="22"/>
     </row>
     <row r="58" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B58" s="2">
+      <c r="B58" s="8">
         <v>6</v>
       </c>
-      <c r="C58" s="3">
-        <v>45992</v>
-      </c>
-      <c r="D58" s="4"/>
-      <c r="E58" s="4"/>
-      <c r="F58" s="5">
+      <c r="C58" s="9">
+        <v>45994</v>
+      </c>
+      <c r="D58" s="10">
+        <v>0.4375</v>
+      </c>
+      <c r="E58" s="10">
+        <v>0.49305555555555558</v>
+      </c>
+      <c r="F58" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G58" s="12"/>
-      <c r="H58" s="12"/>
-      <c r="I58" s="12"/>
-      <c r="J58" s="12"/>
-      <c r="K58" s="12"/>
+        <v>1.3333333333333339</v>
+      </c>
+      <c r="G58" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H58" s="22"/>
+      <c r="I58" s="22"/>
+      <c r="J58" s="22"/>
+      <c r="K58" s="22"/>
     </row>
     <row r="59" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B59" s="2">
+      <c r="B59" s="8">
         <v>6</v>
       </c>
-      <c r="C59" s="3">
-        <v>45992</v>
-      </c>
-      <c r="D59" s="4"/>
-      <c r="E59" s="4"/>
-      <c r="F59" s="5">
+      <c r="C59" s="9">
+        <v>45994</v>
+      </c>
+      <c r="D59" s="10">
+        <v>0.53125</v>
+      </c>
+      <c r="E59" s="10">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F59" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G59" s="12"/>
-      <c r="H59" s="12"/>
-      <c r="I59" s="12"/>
-      <c r="J59" s="12"/>
-      <c r="K59" s="12"/>
+        <v>4.2500000000000009</v>
+      </c>
+      <c r="G59" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="H59" s="22"/>
+      <c r="I59" s="22"/>
+      <c r="J59" s="22"/>
+      <c r="K59" s="22"/>
     </row>
     <row r="60" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B60" s="2">
+      <c r="B60" s="8">
         <v>6</v>
       </c>
-      <c r="C60" s="3">
-        <v>45992</v>
-      </c>
-      <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
-      <c r="F60" s="5">
+      <c r="C60" s="9">
+        <v>45995</v>
+      </c>
+      <c r="D60" s="10">
+        <v>0.4375</v>
+      </c>
+      <c r="E60" s="10">
+        <v>0.49305555555555558</v>
+      </c>
+      <c r="F60" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G60" s="12"/>
-      <c r="H60" s="12"/>
-      <c r="I60" s="12"/>
-      <c r="J60" s="12"/>
-      <c r="K60" s="12"/>
+        <v>1.3333333333333339</v>
+      </c>
+      <c r="G60" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H60" s="22"/>
+      <c r="I60" s="22"/>
+      <c r="J60" s="22"/>
+      <c r="K60" s="22"/>
     </row>
     <row r="61" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B61" s="2">
+      <c r="B61" s="8">
         <v>6</v>
       </c>
-      <c r="C61" s="3">
-        <v>45992</v>
-      </c>
-      <c r="D61" s="4"/>
-      <c r="E61" s="4"/>
-      <c r="F61" s="5">
+      <c r="C61" s="9">
+        <v>45995</v>
+      </c>
+      <c r="D61" s="10">
+        <v>0.53125</v>
+      </c>
+      <c r="E61" s="10">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F61" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G61" s="12"/>
-      <c r="H61" s="12"/>
-      <c r="I61" s="12"/>
-      <c r="J61" s="12"/>
-      <c r="K61" s="12"/>
+        <v>4.2500000000000009</v>
+      </c>
+      <c r="G61" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="H61" s="22"/>
+      <c r="I61" s="22"/>
+      <c r="J61" s="22"/>
+      <c r="K61" s="22"/>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B62" s="2">
+      <c r="B62" s="8">
         <v>6</v>
       </c>
-      <c r="C62" s="3">
-        <v>45992</v>
-      </c>
-      <c r="D62" s="4"/>
-      <c r="E62" s="4"/>
-      <c r="F62" s="5">
+      <c r="C62" s="9">
+        <v>45996</v>
+      </c>
+      <c r="D62" s="10">
+        <v>0.4375</v>
+      </c>
+      <c r="E62" s="10">
+        <v>0.49305555555555558</v>
+      </c>
+      <c r="F62" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G62" s="12"/>
-      <c r="H62" s="12"/>
-      <c r="I62" s="12"/>
-      <c r="J62" s="12"/>
-      <c r="K62" s="12"/>
+        <v>1.3333333333333339</v>
+      </c>
+      <c r="G62" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H62" s="22"/>
+      <c r="I62" s="22"/>
+      <c r="J62" s="22"/>
+      <c r="K62" s="22"/>
     </row>
     <row r="63" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B63" s="2">
+      <c r="B63" s="8">
         <v>6</v>
       </c>
-      <c r="C63" s="3">
-        <v>45992</v>
-      </c>
-      <c r="D63" s="4"/>
-      <c r="E63" s="4"/>
-      <c r="F63" s="5">
+      <c r="C63" s="9">
+        <v>45996</v>
+      </c>
+      <c r="D63" s="10">
+        <v>0.53125</v>
+      </c>
+      <c r="E63" s="10">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F63" s="11">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G63" s="12"/>
-      <c r="H63" s="12"/>
-      <c r="I63" s="12"/>
-      <c r="J63" s="12"/>
-      <c r="K63" s="12"/>
+        <v>4.2500000000000009</v>
+      </c>
+      <c r="G63" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="H63" s="22"/>
+      <c r="I63" s="22"/>
+      <c r="J63" s="22"/>
+      <c r="K63" s="22"/>
     </row>
     <row r="64" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B64" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C64" s="3">
-        <v>45992</v>
-      </c>
-      <c r="D64" s="4"/>
-      <c r="E64" s="4"/>
+        <v>45998</v>
+      </c>
+      <c r="D64" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="E64" s="4">
+        <v>0.58333333333333337</v>
+      </c>
       <c r="F64" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G64" s="12"/>
+        <v>2.0000000000000009</v>
+      </c>
+      <c r="G64" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="H64" s="12"/>
       <c r="I64" s="12"/>
       <c r="J64" s="12"/>
@@ -2164,18 +2233,24 @@
     </row>
     <row r="65" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B65" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C65" s="3">
-        <v>45992</v>
-      </c>
-      <c r="D65" s="4"/>
-      <c r="E65" s="4"/>
+        <v>45998</v>
+      </c>
+      <c r="D65" s="4">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E65" s="4">
+        <v>0.66666666666666663</v>
+      </c>
       <c r="F65" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G65" s="12"/>
+        <v>1.9999999999999982</v>
+      </c>
+      <c r="G65" s="12" t="s">
+        <v>30</v>
+      </c>
       <c r="H65" s="12"/>
       <c r="I65" s="12"/>
       <c r="J65" s="12"/>
@@ -2183,18 +2258,24 @@
     </row>
     <row r="66" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B66" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C66" s="3">
-        <v>45992</v>
-      </c>
-      <c r="D66" s="4"/>
-      <c r="E66" s="4"/>
+        <v>45999</v>
+      </c>
+      <c r="D66" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E66" s="4">
+        <v>0.45833333333333331</v>
+      </c>
       <c r="F66" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G66" s="12"/>
+        <v>0.99999999999999911</v>
+      </c>
+      <c r="G66" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="H66" s="12"/>
       <c r="I66" s="12"/>
       <c r="J66" s="12"/>
@@ -2202,18 +2283,24 @@
     </row>
     <row r="67" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B67" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C67" s="3">
-        <v>45992</v>
-      </c>
-      <c r="D67" s="4"/>
-      <c r="E67" s="4"/>
+        <v>45999</v>
+      </c>
+      <c r="D67" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="E67" s="4">
+        <v>0.5</v>
+      </c>
       <c r="F67" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G67" s="12"/>
+        <v>1.0000000000000004</v>
+      </c>
+      <c r="G67" s="12" t="s">
+        <v>14</v>
+      </c>
       <c r="H67" s="12"/>
       <c r="I67" s="12"/>
       <c r="J67" s="12"/>
@@ -2221,7 +2308,7 @@
     </row>
     <row r="68" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B68" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C68" s="3">
         <v>45992</v>
@@ -2240,56 +2327,14 @@
     </row>
   </sheetData>
   <mergeCells count="74">
-    <mergeCell ref="G65:K65"/>
-    <mergeCell ref="G66:K66"/>
-    <mergeCell ref="G67:K67"/>
-    <mergeCell ref="G68:K68"/>
-    <mergeCell ref="G60:K60"/>
-    <mergeCell ref="G61:K61"/>
-    <mergeCell ref="G62:K62"/>
-    <mergeCell ref="G63:K63"/>
-    <mergeCell ref="G64:K64"/>
-    <mergeCell ref="G55:K55"/>
-    <mergeCell ref="G56:K56"/>
-    <mergeCell ref="G57:K57"/>
-    <mergeCell ref="G58:K58"/>
-    <mergeCell ref="G59:K59"/>
-    <mergeCell ref="G45:K45"/>
-    <mergeCell ref="G40:K40"/>
-    <mergeCell ref="G41:K41"/>
-    <mergeCell ref="G42:K42"/>
-    <mergeCell ref="G43:K43"/>
-    <mergeCell ref="G44:K44"/>
-    <mergeCell ref="G35:K35"/>
-    <mergeCell ref="G36:K36"/>
-    <mergeCell ref="G37:K37"/>
-    <mergeCell ref="G38:K38"/>
-    <mergeCell ref="G39:K39"/>
-    <mergeCell ref="G30:K30"/>
-    <mergeCell ref="G31:K31"/>
-    <mergeCell ref="G32:K32"/>
-    <mergeCell ref="G33:K33"/>
-    <mergeCell ref="G34:K34"/>
-    <mergeCell ref="U5:V5"/>
-    <mergeCell ref="U6:V7"/>
-    <mergeCell ref="G8:K8"/>
-    <mergeCell ref="S5:T5"/>
-    <mergeCell ref="S6:T7"/>
-    <mergeCell ref="S8:T8"/>
-    <mergeCell ref="G3:K3"/>
-    <mergeCell ref="G4:K4"/>
-    <mergeCell ref="G5:K5"/>
-    <mergeCell ref="G6:K6"/>
-    <mergeCell ref="G7:K7"/>
-    <mergeCell ref="G18:K18"/>
-    <mergeCell ref="G29:K29"/>
-    <mergeCell ref="G21:K21"/>
-    <mergeCell ref="G22:K22"/>
-    <mergeCell ref="G23:K23"/>
-    <mergeCell ref="G24:K24"/>
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="G26:K26"/>
-    <mergeCell ref="G19:K19"/>
+    <mergeCell ref="G52:K52"/>
+    <mergeCell ref="G53:K53"/>
+    <mergeCell ref="G54:K54"/>
+    <mergeCell ref="G47:K47"/>
+    <mergeCell ref="G48:K48"/>
+    <mergeCell ref="G49:K49"/>
+    <mergeCell ref="G50:K50"/>
+    <mergeCell ref="G51:K51"/>
     <mergeCell ref="G46:K46"/>
     <mergeCell ref="S9:T9"/>
     <mergeCell ref="U8:V8"/>
@@ -2306,14 +2351,56 @@
     <mergeCell ref="G15:K15"/>
     <mergeCell ref="G16:K16"/>
     <mergeCell ref="G17:K17"/>
-    <mergeCell ref="G52:K52"/>
-    <mergeCell ref="G53:K53"/>
-    <mergeCell ref="G54:K54"/>
-    <mergeCell ref="G47:K47"/>
-    <mergeCell ref="G48:K48"/>
-    <mergeCell ref="G49:K49"/>
-    <mergeCell ref="G50:K50"/>
-    <mergeCell ref="G51:K51"/>
+    <mergeCell ref="G18:K18"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="G21:K21"/>
+    <mergeCell ref="G22:K22"/>
+    <mergeCell ref="G23:K23"/>
+    <mergeCell ref="G24:K24"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="G26:K26"/>
+    <mergeCell ref="G19:K19"/>
+    <mergeCell ref="G3:K3"/>
+    <mergeCell ref="G4:K4"/>
+    <mergeCell ref="G5:K5"/>
+    <mergeCell ref="G6:K6"/>
+    <mergeCell ref="G7:K7"/>
+    <mergeCell ref="U5:V5"/>
+    <mergeCell ref="U6:V7"/>
+    <mergeCell ref="G8:K8"/>
+    <mergeCell ref="S5:T5"/>
+    <mergeCell ref="S6:T7"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="G30:K30"/>
+    <mergeCell ref="G31:K31"/>
+    <mergeCell ref="G32:K32"/>
+    <mergeCell ref="G33:K33"/>
+    <mergeCell ref="G34:K34"/>
+    <mergeCell ref="G35:K35"/>
+    <mergeCell ref="G36:K36"/>
+    <mergeCell ref="G37:K37"/>
+    <mergeCell ref="G38:K38"/>
+    <mergeCell ref="G39:K39"/>
+    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="G40:K40"/>
+    <mergeCell ref="G41:K41"/>
+    <mergeCell ref="G42:K42"/>
+    <mergeCell ref="G43:K43"/>
+    <mergeCell ref="G44:K44"/>
+    <mergeCell ref="G55:K55"/>
+    <mergeCell ref="G56:K56"/>
+    <mergeCell ref="G57:K57"/>
+    <mergeCell ref="G58:K58"/>
+    <mergeCell ref="G59:K59"/>
+    <mergeCell ref="G65:K65"/>
+    <mergeCell ref="G66:K66"/>
+    <mergeCell ref="G67:K67"/>
+    <mergeCell ref="G68:K68"/>
+    <mergeCell ref="G60:K60"/>
+    <mergeCell ref="G61:K61"/>
+    <mergeCell ref="G62:K62"/>
+    <mergeCell ref="G63:K63"/>
+    <mergeCell ref="G64:K64"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="U6" r:id="rId1" xr:uid="{C20C1F99-1D02-49D1-A4F0-3A6675C39A16}"/>

</xml_diff>

<commit_message>
updated cad files and hours
</commit_message>
<xml_diff>
--- a/Documentation/F25/JustinHours.xlsx
+++ b/Documentation/F25/JustinHours.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juxin\Documents\MIDI-Projects\Documentation\F25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFF3D67D-F491-4735-BD99-C5E3B7F35E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B42418F-0EFA-4BCA-8751-78BB5B212A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="40">
   <si>
     <t>Date</t>
   </si>
@@ -138,6 +138,24 @@
   </si>
   <si>
     <t>Fret solenoid terminations and installation</t>
+  </si>
+  <si>
+    <t>Fret solenoid installation</t>
+  </si>
+  <si>
+    <t>Plucking solenoid terminations and installation</t>
+  </si>
+  <si>
+    <t>I2C troubleshooting</t>
+  </si>
+  <si>
+    <t>Fret assembly</t>
+  </si>
+  <si>
+    <t>Documentation</t>
+  </si>
+  <si>
+    <t>Presentation practice</t>
   </si>
 </sst>
 </file>
@@ -292,6 +310,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -306,9 +327,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -591,7 +609,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42FD6328-9B9A-4BF0-A590-87E294C13DA0}">
-  <dimension ref="B3:X79"/>
+  <dimension ref="B3:X94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="1"/>
@@ -715,10 +733,10 @@
         <v>9</v>
       </c>
       <c r="T6" s="12"/>
-      <c r="U6" s="20" t="s">
+      <c r="U6" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="V6" s="21"/>
+      <c r="V6" s="22"/>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
@@ -746,8 +764,8 @@
       <c r="K7" s="12"/>
       <c r="S7" s="12"/>
       <c r="T7" s="12"/>
-      <c r="U7" s="21"/>
-      <c r="V7" s="21"/>
+      <c r="U7" s="22"/>
+      <c r="V7" s="22"/>
     </row>
     <row r="8" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
@@ -773,14 +791,14 @@
       <c r="I8" s="12"/>
       <c r="J8" s="12"/>
       <c r="K8" s="12"/>
-      <c r="S8" s="22" t="s">
+      <c r="S8" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="T8" s="22"/>
-      <c r="U8" s="22">
+      <c r="T8" s="17"/>
+      <c r="U8" s="17">
         <v>430450810</v>
       </c>
-      <c r="V8" s="22"/>
+      <c r="V8" s="17"/>
     </row>
     <row r="9" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
@@ -806,14 +824,14 @@
       <c r="I9" s="12"/>
       <c r="J9" s="12"/>
       <c r="K9" s="12"/>
-      <c r="S9" s="22" t="s">
+      <c r="S9" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="T9" s="22"/>
-      <c r="U9" s="22">
+      <c r="T9" s="17"/>
+      <c r="U9" s="17">
         <v>430450200</v>
       </c>
-      <c r="V9" s="22"/>
+      <c r="V9" s="17"/>
     </row>
     <row r="10" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
@@ -1304,13 +1322,13 @@
         <f t="shared" si="0"/>
         <v>2.333333333333333</v>
       </c>
-      <c r="G27" s="17" t="s">
+      <c r="G27" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H27" s="18"/>
-      <c r="I27" s="18"/>
-      <c r="J27" s="18"/>
-      <c r="K27" s="19"/>
+      <c r="H27" s="19"/>
+      <c r="I27" s="19"/>
+      <c r="J27" s="19"/>
+      <c r="K27" s="20"/>
     </row>
     <row r="28" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B28" s="2">
@@ -1329,13 +1347,13 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G28" s="17" t="s">
+      <c r="G28" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="18"/>
-      <c r="K28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="20"/>
     </row>
     <row r="29" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B29" s="2">
@@ -1354,13 +1372,13 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G29" s="17" t="s">
+      <c r="G29" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H29" s="18"/>
-      <c r="I29" s="18"/>
-      <c r="J29" s="18"/>
-      <c r="K29" s="19"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="19"/>
+      <c r="J29" s="19"/>
+      <c r="K29" s="20"/>
     </row>
     <row r="30" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B30" s="2">
@@ -1379,13 +1397,13 @@
         <f t="shared" ref="F30:F45" si="1">ABS((E30-D30)*24)</f>
         <v>3</v>
       </c>
-      <c r="G30" s="17" t="s">
+      <c r="G30" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="18"/>
-      <c r="I30" s="18"/>
-      <c r="J30" s="18"/>
-      <c r="K30" s="19"/>
+      <c r="H30" s="19"/>
+      <c r="I30" s="19"/>
+      <c r="J30" s="19"/>
+      <c r="K30" s="20"/>
     </row>
     <row r="31" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B31" s="2">
@@ -1404,13 +1422,13 @@
         <f t="shared" si="1"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G31" s="17" t="s">
+      <c r="G31" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
-      <c r="J31" s="18"/>
-      <c r="K31" s="19"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="19"/>
+      <c r="K31" s="20"/>
     </row>
     <row r="32" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B32" s="8">
@@ -2001,7 +2019,7 @@
         <v>0.61805555555555558</v>
       </c>
       <c r="F55" s="11">
-        <f t="shared" ref="F55:F70" si="3">ABS((E55-D55)*24)</f>
+        <f t="shared" ref="F55:F82" si="3">ABS((E55-D55)*24)</f>
         <v>1.1666666666666679</v>
       </c>
       <c r="G55" s="13" t="s">
@@ -2391,11 +2409,22 @@
       <c r="B71" s="2">
         <v>7</v>
       </c>
-      <c r="C71" s="3"/>
-      <c r="D71" s="4"/>
-      <c r="E71" s="4"/>
-      <c r="F71" s="5"/>
-      <c r="G71" s="12"/>
+      <c r="C71" s="3">
+        <v>46001</v>
+      </c>
+      <c r="D71" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E71" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="F71" s="5">
+        <f t="shared" si="3"/>
+        <v>0.99999999999999911</v>
+      </c>
+      <c r="G71" s="12" t="s">
+        <v>34</v>
+      </c>
       <c r="H71" s="12"/>
       <c r="I71" s="12"/>
       <c r="J71" s="12"/>
@@ -2405,11 +2434,22 @@
       <c r="B72" s="2">
         <v>7</v>
       </c>
-      <c r="C72" s="3"/>
-      <c r="D72" s="4"/>
-      <c r="E72" s="4"/>
-      <c r="F72" s="5"/>
-      <c r="G72" s="12"/>
+      <c r="C72" s="3">
+        <v>46001</v>
+      </c>
+      <c r="D72" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="E72" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="F72" s="5">
+        <f t="shared" si="3"/>
+        <v>1.0000000000000004</v>
+      </c>
+      <c r="G72" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="H72" s="12"/>
       <c r="I72" s="12"/>
       <c r="J72" s="12"/>
@@ -2419,109 +2459,448 @@
       <c r="B73" s="2">
         <v>7</v>
       </c>
-      <c r="C73" s="3"/>
-      <c r="D73" s="4"/>
-      <c r="E73" s="4"/>
-      <c r="F73" s="5"/>
-      <c r="G73" s="12"/>
+      <c r="C73" s="3">
+        <v>46001</v>
+      </c>
+      <c r="D73" s="4">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="E73" s="4">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="F73" s="5">
+        <f t="shared" si="3"/>
+        <v>3.4999999999999982</v>
+      </c>
+      <c r="G73" s="12" t="s">
+        <v>35</v>
+      </c>
       <c r="H73" s="12"/>
       <c r="I73" s="12"/>
       <c r="J73" s="12"/>
       <c r="K73" s="12"/>
     </row>
     <row r="74" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B74" s="2"/>
-      <c r="C74" s="3"/>
-      <c r="D74" s="4"/>
-      <c r="E74" s="4"/>
-      <c r="F74" s="5"/>
-      <c r="G74" s="12"/>
+      <c r="B74" s="2">
+        <v>7</v>
+      </c>
+      <c r="C74" s="3">
+        <v>46001</v>
+      </c>
+      <c r="D74" s="4">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="E74" s="4">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F74" s="5">
+        <f t="shared" si="3"/>
+        <v>1.0000000000000018</v>
+      </c>
+      <c r="G74" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="H74" s="12"/>
       <c r="I74" s="12"/>
       <c r="J74" s="12"/>
       <c r="K74" s="12"/>
     </row>
     <row r="75" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B75" s="2"/>
-      <c r="C75" s="3"/>
-      <c r="D75" s="4"/>
-      <c r="E75" s="4"/>
-      <c r="F75" s="5"/>
-      <c r="G75" s="12"/>
+      <c r="B75" s="2">
+        <v>7</v>
+      </c>
+      <c r="C75" s="3">
+        <v>46002</v>
+      </c>
+      <c r="D75" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E75" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="F75" s="5">
+        <f t="shared" si="3"/>
+        <v>1.9999999999999996</v>
+      </c>
+      <c r="G75" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="H75" s="12"/>
       <c r="I75" s="12"/>
       <c r="J75" s="12"/>
       <c r="K75" s="12"/>
     </row>
     <row r="76" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B76" s="2"/>
-      <c r="C76" s="3"/>
-      <c r="D76" s="4"/>
-      <c r="E76" s="4"/>
-      <c r="F76" s="5"/>
-      <c r="G76" s="12"/>
+      <c r="B76" s="2">
+        <v>7</v>
+      </c>
+      <c r="C76" s="3">
+        <v>46002</v>
+      </c>
+      <c r="D76" s="4">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E76" s="4">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="F76" s="5">
+        <f t="shared" si="3"/>
+        <v>2.5000000000000018</v>
+      </c>
+      <c r="G76" s="12" t="s">
+        <v>37</v>
+      </c>
       <c r="H76" s="12"/>
       <c r="I76" s="12"/>
       <c r="J76" s="12"/>
       <c r="K76" s="12"/>
     </row>
     <row r="77" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B77" s="2"/>
-      <c r="C77" s="3"/>
-      <c r="D77" s="4"/>
-      <c r="E77" s="4"/>
-      <c r="F77" s="5"/>
-      <c r="G77" s="12"/>
+      <c r="B77" s="2">
+        <v>7</v>
+      </c>
+      <c r="C77" s="3">
+        <v>46003</v>
+      </c>
+      <c r="D77" s="4">
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="E77" s="4">
+        <v>0.51041666666666663</v>
+      </c>
+      <c r="F77" s="5">
+        <f t="shared" si="3"/>
+        <v>1.583333333333333</v>
+      </c>
+      <c r="G77" s="12" t="s">
+        <v>14</v>
+      </c>
       <c r="H77" s="12"/>
       <c r="I77" s="12"/>
       <c r="J77" s="12"/>
       <c r="K77" s="12"/>
     </row>
     <row r="78" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B78" s="2"/>
-      <c r="C78" s="3"/>
-      <c r="D78" s="4"/>
-      <c r="E78" s="4"/>
-      <c r="F78" s="5"/>
-      <c r="G78" s="12"/>
+      <c r="B78" s="2">
+        <v>7</v>
+      </c>
+      <c r="C78" s="3">
+        <v>46003</v>
+      </c>
+      <c r="D78" s="4">
+        <v>0.53125</v>
+      </c>
+      <c r="E78" s="4">
+        <v>0.6875</v>
+      </c>
+      <c r="F78" s="5">
+        <f t="shared" si="3"/>
+        <v>3.75</v>
+      </c>
+      <c r="G78" s="12" t="s">
+        <v>36</v>
+      </c>
       <c r="H78" s="12"/>
       <c r="I78" s="12"/>
       <c r="J78" s="12"/>
       <c r="K78" s="12"/>
     </row>
     <row r="79" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B79" s="2"/>
-      <c r="C79" s="3"/>
-      <c r="D79" s="4"/>
-      <c r="E79" s="4"/>
-      <c r="F79" s="5"/>
-      <c r="G79" s="12"/>
+      <c r="B79" s="2">
+        <v>8</v>
+      </c>
+      <c r="C79" s="3">
+        <v>46005</v>
+      </c>
+      <c r="D79" s="4">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E79" s="4">
+        <v>0.6875</v>
+      </c>
+      <c r="F79" s="5">
+        <f t="shared" si="3"/>
+        <v>3.5000000000000009</v>
+      </c>
+      <c r="G79" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="H79" s="12"/>
       <c r="I79" s="12"/>
       <c r="J79" s="12"/>
       <c r="K79" s="12"/>
     </row>
+    <row r="80" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B80" s="2">
+        <v>8</v>
+      </c>
+      <c r="C80" s="3">
+        <v>46006</v>
+      </c>
+      <c r="D80" s="4">
+        <v>0.375</v>
+      </c>
+      <c r="E80" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="F80" s="5">
+        <f t="shared" si="3"/>
+        <v>3</v>
+      </c>
+      <c r="G80" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H80" s="12"/>
+      <c r="I80" s="12"/>
+      <c r="J80" s="12"/>
+      <c r="K80" s="12"/>
+    </row>
+    <row r="81" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B81" s="2">
+        <v>8</v>
+      </c>
+      <c r="C81" s="3">
+        <v>46006</v>
+      </c>
+      <c r="D81" s="4">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E81" s="4">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="F81" s="5">
+        <f t="shared" si="3"/>
+        <v>1.7500000000000018</v>
+      </c>
+      <c r="G81" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="H81" s="12"/>
+      <c r="I81" s="12"/>
+      <c r="J81" s="12"/>
+      <c r="K81" s="12"/>
+    </row>
+    <row r="82" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B82" s="2">
+        <v>8</v>
+      </c>
+      <c r="C82" s="3">
+        <v>46006</v>
+      </c>
+      <c r="D82" s="4">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="E82" s="4">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F82" s="5">
+        <f t="shared" si="3"/>
+        <v>2.25</v>
+      </c>
+      <c r="G82" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="H82" s="12"/>
+      <c r="I82" s="12"/>
+      <c r="J82" s="12"/>
+      <c r="K82" s="12"/>
+    </row>
+    <row r="83" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B83" s="2"/>
+      <c r="C83" s="3"/>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4"/>
+      <c r="F83" s="5"/>
+      <c r="G83" s="12"/>
+      <c r="H83" s="12"/>
+      <c r="I83" s="12"/>
+      <c r="J83" s="12"/>
+      <c r="K83" s="12"/>
+    </row>
+    <row r="84" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B84" s="2"/>
+      <c r="C84" s="3"/>
+      <c r="D84" s="4"/>
+      <c r="E84" s="4"/>
+      <c r="F84" s="5"/>
+      <c r="G84" s="12"/>
+      <c r="H84" s="12"/>
+      <c r="I84" s="12"/>
+      <c r="J84" s="12"/>
+      <c r="K84" s="12"/>
+    </row>
+    <row r="85" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B85" s="2"/>
+      <c r="C85" s="3"/>
+      <c r="D85" s="4"/>
+      <c r="E85" s="4"/>
+      <c r="F85" s="5"/>
+      <c r="G85" s="12"/>
+      <c r="H85" s="12"/>
+      <c r="I85" s="12"/>
+      <c r="J85" s="12"/>
+      <c r="K85" s="12"/>
+    </row>
+    <row r="86" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B86" s="2"/>
+      <c r="C86" s="3"/>
+      <c r="D86" s="4"/>
+      <c r="E86" s="4"/>
+      <c r="F86" s="5"/>
+      <c r="G86" s="12"/>
+      <c r="H86" s="12"/>
+      <c r="I86" s="12"/>
+      <c r="J86" s="12"/>
+      <c r="K86" s="12"/>
+    </row>
+    <row r="87" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B87" s="2"/>
+      <c r="C87" s="3"/>
+      <c r="D87" s="4"/>
+      <c r="E87" s="4"/>
+      <c r="F87" s="5"/>
+      <c r="G87" s="12"/>
+      <c r="H87" s="12"/>
+      <c r="I87" s="12"/>
+      <c r="J87" s="12"/>
+      <c r="K87" s="12"/>
+    </row>
+    <row r="88" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B88" s="2"/>
+      <c r="C88" s="3"/>
+      <c r="D88" s="4"/>
+      <c r="E88" s="4"/>
+      <c r="F88" s="5"/>
+      <c r="G88" s="12"/>
+      <c r="H88" s="12"/>
+      <c r="I88" s="12"/>
+      <c r="J88" s="12"/>
+      <c r="K88" s="12"/>
+    </row>
+    <row r="89" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B89" s="2"/>
+      <c r="C89" s="3"/>
+      <c r="D89" s="4"/>
+      <c r="E89" s="4"/>
+      <c r="F89" s="5"/>
+      <c r="G89" s="12"/>
+      <c r="H89" s="12"/>
+      <c r="I89" s="12"/>
+      <c r="J89" s="12"/>
+      <c r="K89" s="12"/>
+    </row>
+    <row r="90" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B90" s="2"/>
+      <c r="C90" s="3"/>
+      <c r="D90" s="4"/>
+      <c r="E90" s="4"/>
+      <c r="F90" s="5"/>
+      <c r="G90" s="12"/>
+      <c r="H90" s="12"/>
+      <c r="I90" s="12"/>
+      <c r="J90" s="12"/>
+      <c r="K90" s="12"/>
+    </row>
+    <row r="91" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B91" s="2"/>
+      <c r="C91" s="3"/>
+      <c r="D91" s="4"/>
+      <c r="E91" s="4"/>
+      <c r="F91" s="5"/>
+      <c r="G91" s="12"/>
+      <c r="H91" s="12"/>
+      <c r="I91" s="12"/>
+      <c r="J91" s="12"/>
+      <c r="K91" s="12"/>
+    </row>
+    <row r="92" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B92" s="2"/>
+      <c r="C92" s="3"/>
+      <c r="D92" s="4"/>
+      <c r="E92" s="4"/>
+      <c r="F92" s="5"/>
+      <c r="G92" s="12"/>
+      <c r="H92" s="12"/>
+      <c r="I92" s="12"/>
+      <c r="J92" s="12"/>
+      <c r="K92" s="12"/>
+    </row>
+    <row r="93" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B93" s="2"/>
+      <c r="C93" s="3"/>
+      <c r="D93" s="4"/>
+      <c r="E93" s="4"/>
+      <c r="F93" s="5"/>
+      <c r="G93" s="12"/>
+      <c r="H93" s="12"/>
+      <c r="I93" s="12"/>
+      <c r="J93" s="12"/>
+      <c r="K93" s="12"/>
+    </row>
+    <row r="94" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B94" s="2"/>
+      <c r="C94" s="3"/>
+      <c r="D94" s="4"/>
+      <c r="E94" s="4"/>
+      <c r="F94" s="5"/>
+      <c r="G94" s="12"/>
+      <c r="H94" s="12"/>
+      <c r="I94" s="12"/>
+      <c r="J94" s="12"/>
+      <c r="K94" s="12"/>
+    </row>
   </sheetData>
-  <mergeCells count="85">
-    <mergeCell ref="G79:K79"/>
-    <mergeCell ref="G74:K74"/>
-    <mergeCell ref="G75:K75"/>
-    <mergeCell ref="G76:K76"/>
-    <mergeCell ref="G77:K77"/>
-    <mergeCell ref="G78:K78"/>
-    <mergeCell ref="G69:K69"/>
-    <mergeCell ref="G70:K70"/>
-    <mergeCell ref="G71:K71"/>
-    <mergeCell ref="G72:K72"/>
-    <mergeCell ref="G73:K73"/>
-    <mergeCell ref="G52:K52"/>
-    <mergeCell ref="G53:K53"/>
-    <mergeCell ref="G54:K54"/>
-    <mergeCell ref="G47:K47"/>
-    <mergeCell ref="G48:K48"/>
-    <mergeCell ref="G49:K49"/>
-    <mergeCell ref="G50:K50"/>
-    <mergeCell ref="G51:K51"/>
+  <mergeCells count="100">
+    <mergeCell ref="G65:K65"/>
+    <mergeCell ref="G66:K66"/>
+    <mergeCell ref="G67:K67"/>
+    <mergeCell ref="G68:K68"/>
+    <mergeCell ref="G60:K60"/>
+    <mergeCell ref="G61:K61"/>
+    <mergeCell ref="G62:K62"/>
+    <mergeCell ref="G63:K63"/>
+    <mergeCell ref="G64:K64"/>
+    <mergeCell ref="G55:K55"/>
+    <mergeCell ref="G56:K56"/>
+    <mergeCell ref="G57:K57"/>
+    <mergeCell ref="G58:K58"/>
+    <mergeCell ref="G59:K59"/>
+    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="G40:K40"/>
+    <mergeCell ref="G41:K41"/>
+    <mergeCell ref="G42:K42"/>
+    <mergeCell ref="G43:K43"/>
+    <mergeCell ref="G44:K44"/>
+    <mergeCell ref="G35:K35"/>
+    <mergeCell ref="G36:K36"/>
+    <mergeCell ref="G37:K37"/>
+    <mergeCell ref="G38:K38"/>
+    <mergeCell ref="G39:K39"/>
+    <mergeCell ref="G30:K30"/>
+    <mergeCell ref="G31:K31"/>
+    <mergeCell ref="G32:K32"/>
+    <mergeCell ref="G33:K33"/>
+    <mergeCell ref="G34:K34"/>
+    <mergeCell ref="U5:V5"/>
+    <mergeCell ref="U6:V7"/>
+    <mergeCell ref="G8:K8"/>
+    <mergeCell ref="S5:T5"/>
+    <mergeCell ref="S6:T7"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="G3:K3"/>
+    <mergeCell ref="G4:K4"/>
+    <mergeCell ref="G5:K5"/>
+    <mergeCell ref="G6:K6"/>
+    <mergeCell ref="G7:K7"/>
+    <mergeCell ref="G18:K18"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="G21:K21"/>
+    <mergeCell ref="G22:K22"/>
+    <mergeCell ref="G23:K23"/>
+    <mergeCell ref="G24:K24"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="G26:K26"/>
+    <mergeCell ref="G19:K19"/>
     <mergeCell ref="G46:K46"/>
     <mergeCell ref="S9:T9"/>
     <mergeCell ref="U8:V8"/>
@@ -2538,56 +2917,40 @@
     <mergeCell ref="G15:K15"/>
     <mergeCell ref="G16:K16"/>
     <mergeCell ref="G17:K17"/>
-    <mergeCell ref="G18:K18"/>
-    <mergeCell ref="G29:K29"/>
-    <mergeCell ref="G21:K21"/>
-    <mergeCell ref="G22:K22"/>
-    <mergeCell ref="G23:K23"/>
-    <mergeCell ref="G24:K24"/>
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="G26:K26"/>
-    <mergeCell ref="G19:K19"/>
-    <mergeCell ref="G3:K3"/>
-    <mergeCell ref="G4:K4"/>
-    <mergeCell ref="G5:K5"/>
-    <mergeCell ref="G6:K6"/>
-    <mergeCell ref="G7:K7"/>
-    <mergeCell ref="U5:V5"/>
-    <mergeCell ref="U6:V7"/>
-    <mergeCell ref="G8:K8"/>
-    <mergeCell ref="S5:T5"/>
-    <mergeCell ref="S6:T7"/>
-    <mergeCell ref="S8:T8"/>
-    <mergeCell ref="G30:K30"/>
-    <mergeCell ref="G31:K31"/>
-    <mergeCell ref="G32:K32"/>
-    <mergeCell ref="G33:K33"/>
-    <mergeCell ref="G34:K34"/>
-    <mergeCell ref="G35:K35"/>
-    <mergeCell ref="G36:K36"/>
-    <mergeCell ref="G37:K37"/>
-    <mergeCell ref="G38:K38"/>
-    <mergeCell ref="G39:K39"/>
-    <mergeCell ref="G45:K45"/>
-    <mergeCell ref="G40:K40"/>
-    <mergeCell ref="G41:K41"/>
-    <mergeCell ref="G42:K42"/>
-    <mergeCell ref="G43:K43"/>
-    <mergeCell ref="G44:K44"/>
-    <mergeCell ref="G55:K55"/>
-    <mergeCell ref="G56:K56"/>
-    <mergeCell ref="G57:K57"/>
-    <mergeCell ref="G58:K58"/>
-    <mergeCell ref="G59:K59"/>
-    <mergeCell ref="G65:K65"/>
-    <mergeCell ref="G66:K66"/>
-    <mergeCell ref="G67:K67"/>
-    <mergeCell ref="G68:K68"/>
-    <mergeCell ref="G60:K60"/>
-    <mergeCell ref="G61:K61"/>
-    <mergeCell ref="G62:K62"/>
-    <mergeCell ref="G63:K63"/>
-    <mergeCell ref="G64:K64"/>
+    <mergeCell ref="G52:K52"/>
+    <mergeCell ref="G53:K53"/>
+    <mergeCell ref="G54:K54"/>
+    <mergeCell ref="G47:K47"/>
+    <mergeCell ref="G48:K48"/>
+    <mergeCell ref="G49:K49"/>
+    <mergeCell ref="G50:K50"/>
+    <mergeCell ref="G51:K51"/>
+    <mergeCell ref="G69:K69"/>
+    <mergeCell ref="G70:K70"/>
+    <mergeCell ref="G71:K71"/>
+    <mergeCell ref="G72:K72"/>
+    <mergeCell ref="G73:K73"/>
+    <mergeCell ref="G79:K79"/>
+    <mergeCell ref="G74:K74"/>
+    <mergeCell ref="G75:K75"/>
+    <mergeCell ref="G76:K76"/>
+    <mergeCell ref="G77:K77"/>
+    <mergeCell ref="G78:K78"/>
+    <mergeCell ref="G80:K80"/>
+    <mergeCell ref="G81:K81"/>
+    <mergeCell ref="G82:K82"/>
+    <mergeCell ref="G83:K83"/>
+    <mergeCell ref="G84:K84"/>
+    <mergeCell ref="G85:K85"/>
+    <mergeCell ref="G86:K86"/>
+    <mergeCell ref="G87:K87"/>
+    <mergeCell ref="G88:K88"/>
+    <mergeCell ref="G89:K89"/>
+    <mergeCell ref="G90:K90"/>
+    <mergeCell ref="G91:K91"/>
+    <mergeCell ref="G92:K92"/>
+    <mergeCell ref="G93:K93"/>
+    <mergeCell ref="G94:K94"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="U6" r:id="rId1" xr:uid="{C20C1F99-1D02-49D1-A4F0-3A6675C39A16}"/>

</xml_diff>

<commit_message>
made pdfs for final report
</commit_message>
<xml_diff>
--- a/Documentation/F25/JustinHours.xlsx
+++ b/Documentation/F25/JustinHours.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juxin\Documents\MIDI-Projects\Documentation\F25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21AA93F7-BD72-4167-B392-53B96FE93F6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A44F6B1E-B4CB-4D92-8CE4-E178B9B4FF18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="2625" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="F25" sheetId="6" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="42">
   <si>
     <t>Date</t>
   </si>
@@ -159,6 +159,9 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Cable Making</t>
   </si>
 </sst>
 </file>
@@ -313,6 +316,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -327,9 +333,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -736,10 +739,10 @@
         <v>9</v>
       </c>
       <c r="T6" s="12"/>
-      <c r="U6" s="20" t="s">
+      <c r="U6" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="V6" s="21"/>
+      <c r="V6" s="22"/>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
@@ -767,8 +770,8 @@
       <c r="K7" s="12"/>
       <c r="S7" s="12"/>
       <c r="T7" s="12"/>
-      <c r="U7" s="21"/>
-      <c r="V7" s="21"/>
+      <c r="U7" s="22"/>
+      <c r="V7" s="22"/>
     </row>
     <row r="8" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
@@ -794,14 +797,14 @@
       <c r="I8" s="12"/>
       <c r="J8" s="12"/>
       <c r="K8" s="12"/>
-      <c r="S8" s="22" t="s">
+      <c r="S8" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="T8" s="22"/>
-      <c r="U8" s="22">
+      <c r="T8" s="17"/>
+      <c r="U8" s="17">
         <v>430450810</v>
       </c>
-      <c r="V8" s="22"/>
+      <c r="V8" s="17"/>
     </row>
     <row r="9" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
@@ -827,14 +830,14 @@
       <c r="I9" s="12"/>
       <c r="J9" s="12"/>
       <c r="K9" s="12"/>
-      <c r="S9" s="22" t="s">
+      <c r="S9" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="T9" s="22"/>
-      <c r="U9" s="22">
+      <c r="T9" s="17"/>
+      <c r="U9" s="17">
         <v>430450200</v>
       </c>
-      <c r="V9" s="22"/>
+      <c r="V9" s="17"/>
     </row>
     <row r="10" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
@@ -1325,13 +1328,13 @@
         <f t="shared" si="0"/>
         <v>2.333333333333333</v>
       </c>
-      <c r="G27" s="17" t="s">
+      <c r="G27" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H27" s="18"/>
-      <c r="I27" s="18"/>
-      <c r="J27" s="18"/>
-      <c r="K27" s="19"/>
+      <c r="H27" s="19"/>
+      <c r="I27" s="19"/>
+      <c r="J27" s="19"/>
+      <c r="K27" s="20"/>
     </row>
     <row r="28" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B28" s="2">
@@ -1350,13 +1353,13 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G28" s="17" t="s">
+      <c r="G28" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="18"/>
-      <c r="K28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="20"/>
     </row>
     <row r="29" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B29" s="2">
@@ -1375,13 +1378,13 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G29" s="17" t="s">
+      <c r="G29" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H29" s="18"/>
-      <c r="I29" s="18"/>
-      <c r="J29" s="18"/>
-      <c r="K29" s="19"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="19"/>
+      <c r="J29" s="19"/>
+      <c r="K29" s="20"/>
     </row>
     <row r="30" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B30" s="2">
@@ -1400,13 +1403,13 @@
         <f t="shared" ref="F30:F45" si="1">ABS((E30-D30)*24)</f>
         <v>3</v>
       </c>
-      <c r="G30" s="17" t="s">
+      <c r="G30" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="18"/>
-      <c r="I30" s="18"/>
-      <c r="J30" s="18"/>
-      <c r="K30" s="19"/>
+      <c r="H30" s="19"/>
+      <c r="I30" s="19"/>
+      <c r="J30" s="19"/>
+      <c r="K30" s="20"/>
     </row>
     <row r="31" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B31" s="2">
@@ -1425,13 +1428,13 @@
         <f t="shared" si="1"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G31" s="17" t="s">
+      <c r="G31" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
-      <c r="J31" s="18"/>
-      <c r="K31" s="19"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="19"/>
+      <c r="K31" s="20"/>
     </row>
     <row r="32" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B32" s="8">
@@ -2022,7 +2025,7 @@
         <v>0.61805555555555558</v>
       </c>
       <c r="F55" s="11">
-        <f t="shared" ref="F55:F83" si="3">ABS((E55-D55)*24)</f>
+        <f t="shared" ref="F55:F89" si="3">ABS((E55-D55)*24)</f>
         <v>1.1666666666666679</v>
       </c>
       <c r="G55" s="13" t="s">
@@ -2609,201 +2612,278 @@
       <c r="K78" s="12"/>
     </row>
     <row r="79" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B79" s="2">
+      <c r="B79" s="8">
         <v>8</v>
       </c>
-      <c r="C79" s="3">
+      <c r="C79" s="9">
         <v>46005</v>
       </c>
-      <c r="D79" s="4">
+      <c r="D79" s="10">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E79" s="4">
+      <c r="E79" s="10">
         <v>0.6875</v>
       </c>
-      <c r="F79" s="5">
+      <c r="F79" s="11">
         <f t="shared" si="3"/>
         <v>3.5000000000000009</v>
       </c>
-      <c r="G79" s="12" t="s">
+      <c r="G79" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="H79" s="12"/>
-      <c r="I79" s="12"/>
-      <c r="J79" s="12"/>
-      <c r="K79" s="12"/>
+      <c r="H79" s="13"/>
+      <c r="I79" s="13"/>
+      <c r="J79" s="13"/>
+      <c r="K79" s="13"/>
     </row>
     <row r="80" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B80" s="2">
+      <c r="B80" s="8">
         <v>8</v>
       </c>
-      <c r="C80" s="3">
+      <c r="C80" s="9">
         <v>46006</v>
       </c>
-      <c r="D80" s="4">
+      <c r="D80" s="10">
         <v>0.375</v>
       </c>
-      <c r="E80" s="4">
+      <c r="E80" s="10">
         <v>0.5</v>
       </c>
-      <c r="F80" s="5">
+      <c r="F80" s="11">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="G80" s="12" t="s">
+      <c r="G80" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="H80" s="12"/>
-      <c r="I80" s="12"/>
-      <c r="J80" s="12"/>
-      <c r="K80" s="12"/>
+      <c r="H80" s="13"/>
+      <c r="I80" s="13"/>
+      <c r="J80" s="13"/>
+      <c r="K80" s="13"/>
     </row>
     <row r="81" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B81" s="2">
+      <c r="B81" s="8">
         <v>8</v>
       </c>
-      <c r="C81" s="3">
+      <c r="C81" s="9">
         <v>46006</v>
       </c>
-      <c r="D81" s="4">
+      <c r="D81" s="10">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E81" s="4">
+      <c r="E81" s="10">
         <v>0.61458333333333337</v>
       </c>
-      <c r="F81" s="5">
+      <c r="F81" s="11">
         <f t="shared" si="3"/>
         <v>1.7500000000000018</v>
       </c>
-      <c r="G81" s="12" t="s">
+      <c r="G81" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="H81" s="12"/>
-      <c r="I81" s="12"/>
-      <c r="J81" s="12"/>
-      <c r="K81" s="12"/>
+      <c r="H81" s="13"/>
+      <c r="I81" s="13"/>
+      <c r="J81" s="13"/>
+      <c r="K81" s="13"/>
     </row>
     <row r="82" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B82" s="2">
+      <c r="B82" s="8">
         <v>8</v>
       </c>
-      <c r="C82" s="3">
+      <c r="C82" s="9">
         <v>46006</v>
       </c>
-      <c r="D82" s="4">
+      <c r="D82" s="10">
         <v>0.61458333333333337</v>
       </c>
-      <c r="E82" s="4">
+      <c r="E82" s="10">
         <v>0.70833333333333337</v>
       </c>
-      <c r="F82" s="5">
+      <c r="F82" s="11">
         <f t="shared" si="3"/>
         <v>2.25</v>
       </c>
-      <c r="G82" s="12" t="s">
+      <c r="G82" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="H82" s="12"/>
-      <c r="I82" s="12"/>
-      <c r="J82" s="12"/>
-      <c r="K82" s="12"/>
+      <c r="H82" s="13"/>
+      <c r="I82" s="13"/>
+      <c r="J82" s="13"/>
+      <c r="K82" s="13"/>
     </row>
     <row r="83" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B83" s="2">
+      <c r="B83" s="8">
         <v>8</v>
       </c>
-      <c r="C83" s="3">
+      <c r="C83" s="9">
         <v>46006</v>
       </c>
-      <c r="D83" s="4">
+      <c r="D83" s="10">
         <v>0.875</v>
       </c>
-      <c r="E83" s="4">
+      <c r="E83" s="10">
         <v>0.94791666666666663</v>
       </c>
-      <c r="F83" s="5">
+      <c r="F83" s="11">
         <f t="shared" si="3"/>
         <v>1.7499999999999991</v>
       </c>
-      <c r="G83" s="12" t="s">
+      <c r="G83" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="H83" s="12"/>
-      <c r="I83" s="12"/>
-      <c r="J83" s="12"/>
-      <c r="K83" s="12"/>
+      <c r="H83" s="13"/>
+      <c r="I83" s="13"/>
+      <c r="J83" s="13"/>
+      <c r="K83" s="13"/>
     </row>
     <row r="84" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B84" s="2"/>
-      <c r="C84" s="3"/>
-      <c r="D84" s="4"/>
-      <c r="E84" s="4"/>
-      <c r="F84" s="5"/>
-      <c r="G84" s="12"/>
-      <c r="H84" s="12"/>
-      <c r="I84" s="12"/>
-      <c r="J84" s="12"/>
-      <c r="K84" s="12"/>
+      <c r="B84" s="8">
+        <v>8</v>
+      </c>
+      <c r="C84" s="9">
+        <v>46007</v>
+      </c>
+      <c r="D84" s="10">
+        <v>0.38541666666666669</v>
+      </c>
+      <c r="E84" s="10">
+        <v>0.51041666666666663</v>
+      </c>
+      <c r="F84" s="11">
+        <f t="shared" si="3"/>
+        <v>2.9999999999999987</v>
+      </c>
+      <c r="G84" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="H84" s="13"/>
+      <c r="I84" s="13"/>
+      <c r="J84" s="13"/>
+      <c r="K84" s="13"/>
     </row>
     <row r="85" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B85" s="2"/>
-      <c r="C85" s="3"/>
-      <c r="D85" s="4"/>
-      <c r="E85" s="4"/>
-      <c r="F85" s="5"/>
-      <c r="G85" s="12"/>
-      <c r="H85" s="12"/>
-      <c r="I85" s="12"/>
-      <c r="J85" s="12"/>
-      <c r="K85" s="12"/>
+      <c r="B85" s="8">
+        <v>8</v>
+      </c>
+      <c r="C85" s="9">
+        <v>46007</v>
+      </c>
+      <c r="D85" s="10">
+        <v>0.53125</v>
+      </c>
+      <c r="E85" s="10">
+        <v>0.71875</v>
+      </c>
+      <c r="F85" s="11">
+        <f t="shared" si="3"/>
+        <v>4.5</v>
+      </c>
+      <c r="G85" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="H85" s="13"/>
+      <c r="I85" s="13"/>
+      <c r="J85" s="13"/>
+      <c r="K85" s="13"/>
     </row>
     <row r="86" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B86" s="2"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="4"/>
-      <c r="E86" s="4"/>
-      <c r="F86" s="5"/>
-      <c r="G86" s="12"/>
-      <c r="H86" s="12"/>
-      <c r="I86" s="12"/>
-      <c r="J86" s="12"/>
-      <c r="K86" s="12"/>
+      <c r="B86" s="8">
+        <v>8</v>
+      </c>
+      <c r="C86" s="9">
+        <v>46007</v>
+      </c>
+      <c r="D86" s="10">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="E86" s="10">
+        <v>0.9375</v>
+      </c>
+      <c r="F86" s="11">
+        <f t="shared" si="3"/>
+        <v>3.9999999999999991</v>
+      </c>
+      <c r="G86" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="H86" s="13"/>
+      <c r="I86" s="13"/>
+      <c r="J86" s="13"/>
+      <c r="K86" s="13"/>
     </row>
     <row r="87" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B87" s="2"/>
-      <c r="C87" s="3"/>
-      <c r="D87" s="4"/>
-      <c r="E87" s="4"/>
-      <c r="F87" s="5"/>
-      <c r="G87" s="12"/>
-      <c r="H87" s="12"/>
-      <c r="I87" s="12"/>
-      <c r="J87" s="12"/>
-      <c r="K87" s="12"/>
+      <c r="B87" s="8">
+        <v>8</v>
+      </c>
+      <c r="C87" s="9">
+        <v>46007</v>
+      </c>
+      <c r="D87" s="10">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E87" s="10">
+        <v>0.6875</v>
+      </c>
+      <c r="F87" s="11">
+        <f t="shared" si="3"/>
+        <v>3.5000000000000009</v>
+      </c>
+      <c r="G87" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="H87" s="13"/>
+      <c r="I87" s="13"/>
+      <c r="J87" s="13"/>
+      <c r="K87" s="13"/>
     </row>
     <row r="88" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B88" s="2"/>
-      <c r="C88" s="3"/>
-      <c r="D88" s="4"/>
-      <c r="E88" s="4"/>
-      <c r="F88" s="5"/>
-      <c r="G88" s="12"/>
-      <c r="H88" s="12"/>
-      <c r="I88" s="12"/>
-      <c r="J88" s="12"/>
-      <c r="K88" s="12"/>
+      <c r="B88" s="8">
+        <v>8</v>
+      </c>
+      <c r="C88" s="9">
+        <v>46007</v>
+      </c>
+      <c r="D88" s="10">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="E88" s="10">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="F88" s="11">
+        <f t="shared" si="3"/>
+        <v>1.9999999999999982</v>
+      </c>
+      <c r="G88" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="H88" s="13"/>
+      <c r="I88" s="13"/>
+      <c r="J88" s="13"/>
+      <c r="K88" s="13"/>
     </row>
     <row r="89" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B89" s="2"/>
-      <c r="C89" s="3"/>
-      <c r="D89" s="4"/>
-      <c r="E89" s="4"/>
-      <c r="F89" s="5"/>
-      <c r="G89" s="12"/>
-      <c r="H89" s="12"/>
-      <c r="I89" s="12"/>
-      <c r="J89" s="12"/>
-      <c r="K89" s="12"/>
+      <c r="B89" s="8">
+        <v>8</v>
+      </c>
+      <c r="C89" s="9">
+        <v>46007</v>
+      </c>
+      <c r="D89" s="10">
+        <v>0.92708333333333337</v>
+      </c>
+      <c r="E89" s="10">
+        <v>6.25E-2</v>
+      </c>
+      <c r="F89" s="11">
+        <v>3.25</v>
+      </c>
+      <c r="G89" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="H89" s="13"/>
+      <c r="I89" s="13"/>
+      <c r="J89" s="13"/>
+      <c r="K89" s="13"/>
     </row>
     <row r="90" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B90" s="2"/>
@@ -2870,46 +2950,62 @@
         <v>40</v>
       </c>
       <c r="F95" s="1">
-        <f>SUM(F4:F83)</f>
-        <v>153.19999999999999</v>
+        <f>SUM(F4:F89)</f>
+        <v>173.45</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="100">
-    <mergeCell ref="G90:K90"/>
-    <mergeCell ref="G91:K91"/>
-    <mergeCell ref="G92:K92"/>
-    <mergeCell ref="G93:K93"/>
-    <mergeCell ref="G94:K94"/>
-    <mergeCell ref="G85:K85"/>
-    <mergeCell ref="G86:K86"/>
-    <mergeCell ref="G87:K87"/>
-    <mergeCell ref="G88:K88"/>
-    <mergeCell ref="G89:K89"/>
-    <mergeCell ref="G80:K80"/>
-    <mergeCell ref="G81:K81"/>
-    <mergeCell ref="G82:K82"/>
-    <mergeCell ref="G83:K83"/>
-    <mergeCell ref="G84:K84"/>
-    <mergeCell ref="G79:K79"/>
-    <mergeCell ref="G74:K74"/>
-    <mergeCell ref="G75:K75"/>
-    <mergeCell ref="G76:K76"/>
-    <mergeCell ref="G77:K77"/>
-    <mergeCell ref="G78:K78"/>
-    <mergeCell ref="G69:K69"/>
-    <mergeCell ref="G70:K70"/>
-    <mergeCell ref="G71:K71"/>
-    <mergeCell ref="G72:K72"/>
-    <mergeCell ref="G73:K73"/>
-    <mergeCell ref="G52:K52"/>
-    <mergeCell ref="G53:K53"/>
-    <mergeCell ref="G54:K54"/>
-    <mergeCell ref="G47:K47"/>
-    <mergeCell ref="G48:K48"/>
-    <mergeCell ref="G49:K49"/>
-    <mergeCell ref="G50:K50"/>
-    <mergeCell ref="G51:K51"/>
+    <mergeCell ref="G65:K65"/>
+    <mergeCell ref="G66:K66"/>
+    <mergeCell ref="G67:K67"/>
+    <mergeCell ref="G68:K68"/>
+    <mergeCell ref="G60:K60"/>
+    <mergeCell ref="G61:K61"/>
+    <mergeCell ref="G62:K62"/>
+    <mergeCell ref="G63:K63"/>
+    <mergeCell ref="G64:K64"/>
+    <mergeCell ref="G55:K55"/>
+    <mergeCell ref="G56:K56"/>
+    <mergeCell ref="G57:K57"/>
+    <mergeCell ref="G58:K58"/>
+    <mergeCell ref="G59:K59"/>
+    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="G40:K40"/>
+    <mergeCell ref="G41:K41"/>
+    <mergeCell ref="G42:K42"/>
+    <mergeCell ref="G43:K43"/>
+    <mergeCell ref="G44:K44"/>
+    <mergeCell ref="G35:K35"/>
+    <mergeCell ref="G36:K36"/>
+    <mergeCell ref="G37:K37"/>
+    <mergeCell ref="G38:K38"/>
+    <mergeCell ref="G39:K39"/>
+    <mergeCell ref="G30:K30"/>
+    <mergeCell ref="G31:K31"/>
+    <mergeCell ref="G32:K32"/>
+    <mergeCell ref="G33:K33"/>
+    <mergeCell ref="G34:K34"/>
+    <mergeCell ref="U5:V5"/>
+    <mergeCell ref="U6:V7"/>
+    <mergeCell ref="G8:K8"/>
+    <mergeCell ref="S5:T5"/>
+    <mergeCell ref="S6:T7"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="G3:K3"/>
+    <mergeCell ref="G4:K4"/>
+    <mergeCell ref="G5:K5"/>
+    <mergeCell ref="G6:K6"/>
+    <mergeCell ref="G7:K7"/>
+    <mergeCell ref="G18:K18"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="G21:K21"/>
+    <mergeCell ref="G22:K22"/>
+    <mergeCell ref="G23:K23"/>
+    <mergeCell ref="G24:K24"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="G26:K26"/>
+    <mergeCell ref="G19:K19"/>
     <mergeCell ref="G46:K46"/>
     <mergeCell ref="S9:T9"/>
     <mergeCell ref="U8:V8"/>
@@ -2926,56 +3022,40 @@
     <mergeCell ref="G15:K15"/>
     <mergeCell ref="G16:K16"/>
     <mergeCell ref="G17:K17"/>
-    <mergeCell ref="G18:K18"/>
-    <mergeCell ref="G29:K29"/>
-    <mergeCell ref="G21:K21"/>
-    <mergeCell ref="G22:K22"/>
-    <mergeCell ref="G23:K23"/>
-    <mergeCell ref="G24:K24"/>
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="G26:K26"/>
-    <mergeCell ref="G19:K19"/>
-    <mergeCell ref="G3:K3"/>
-    <mergeCell ref="G4:K4"/>
-    <mergeCell ref="G5:K5"/>
-    <mergeCell ref="G6:K6"/>
-    <mergeCell ref="G7:K7"/>
-    <mergeCell ref="U5:V5"/>
-    <mergeCell ref="U6:V7"/>
-    <mergeCell ref="G8:K8"/>
-    <mergeCell ref="S5:T5"/>
-    <mergeCell ref="S6:T7"/>
-    <mergeCell ref="S8:T8"/>
-    <mergeCell ref="G30:K30"/>
-    <mergeCell ref="G31:K31"/>
-    <mergeCell ref="G32:K32"/>
-    <mergeCell ref="G33:K33"/>
-    <mergeCell ref="G34:K34"/>
-    <mergeCell ref="G35:K35"/>
-    <mergeCell ref="G36:K36"/>
-    <mergeCell ref="G37:K37"/>
-    <mergeCell ref="G38:K38"/>
-    <mergeCell ref="G39:K39"/>
-    <mergeCell ref="G45:K45"/>
-    <mergeCell ref="G40:K40"/>
-    <mergeCell ref="G41:K41"/>
-    <mergeCell ref="G42:K42"/>
-    <mergeCell ref="G43:K43"/>
-    <mergeCell ref="G44:K44"/>
-    <mergeCell ref="G55:K55"/>
-    <mergeCell ref="G56:K56"/>
-    <mergeCell ref="G57:K57"/>
-    <mergeCell ref="G58:K58"/>
-    <mergeCell ref="G59:K59"/>
-    <mergeCell ref="G65:K65"/>
-    <mergeCell ref="G66:K66"/>
-    <mergeCell ref="G67:K67"/>
-    <mergeCell ref="G68:K68"/>
-    <mergeCell ref="G60:K60"/>
-    <mergeCell ref="G61:K61"/>
-    <mergeCell ref="G62:K62"/>
-    <mergeCell ref="G63:K63"/>
-    <mergeCell ref="G64:K64"/>
+    <mergeCell ref="G52:K52"/>
+    <mergeCell ref="G53:K53"/>
+    <mergeCell ref="G54:K54"/>
+    <mergeCell ref="G47:K47"/>
+    <mergeCell ref="G48:K48"/>
+    <mergeCell ref="G49:K49"/>
+    <mergeCell ref="G50:K50"/>
+    <mergeCell ref="G51:K51"/>
+    <mergeCell ref="G69:K69"/>
+    <mergeCell ref="G70:K70"/>
+    <mergeCell ref="G71:K71"/>
+    <mergeCell ref="G72:K72"/>
+    <mergeCell ref="G73:K73"/>
+    <mergeCell ref="G79:K79"/>
+    <mergeCell ref="G74:K74"/>
+    <mergeCell ref="G75:K75"/>
+    <mergeCell ref="G76:K76"/>
+    <mergeCell ref="G77:K77"/>
+    <mergeCell ref="G78:K78"/>
+    <mergeCell ref="G80:K80"/>
+    <mergeCell ref="G81:K81"/>
+    <mergeCell ref="G82:K82"/>
+    <mergeCell ref="G83:K83"/>
+    <mergeCell ref="G84:K84"/>
+    <mergeCell ref="G85:K85"/>
+    <mergeCell ref="G86:K86"/>
+    <mergeCell ref="G87:K87"/>
+    <mergeCell ref="G88:K88"/>
+    <mergeCell ref="G89:K89"/>
+    <mergeCell ref="G90:K90"/>
+    <mergeCell ref="G91:K91"/>
+    <mergeCell ref="G92:K92"/>
+    <mergeCell ref="G93:K93"/>
+    <mergeCell ref="G94:K94"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="U6" r:id="rId1" xr:uid="{C20C1F99-1D02-49D1-A4F0-3A6675C39A16}"/>

</xml_diff>